<commit_message>
maj tableau de synthese
</commit_message>
<xml_diff>
--- a/E5 - Tableau de synthèse AOUZAL Jawad.xlsx
+++ b/E5 - Tableau de synthèse AOUZAL Jawad.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29930"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jawad\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lyceerobertschuman710-my.sharepoint.com/personal/j_aouzal_lprs_fr/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_B009C45352E4F952CA2B341BF94231B0C7EA6DCB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1AB63AA9-F84C-4AB3-A2E9-367745D2559F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,12 +18,28 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E5'!$A$1:$H$35</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="52">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -164,13 +180,19 @@
     <t>19/03/25 au 09/05/25</t>
   </si>
   <si>
-    <t>LPRS</t>
+    <t>Site php LPRS</t>
   </si>
   <si>
     <t>02/09/25 au 10/12/25</t>
   </si>
   <si>
     <t>x</t>
+  </si>
+  <si>
+    <t>Application javafx LPRS</t>
+  </si>
+  <si>
+    <t>10/12/25 au 24/03/26</t>
   </si>
   <si>
     <t>Réalisations en milieu professionnel en cours de première année</t>
@@ -201,7 +223,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="13">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -636,7 +658,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -719,44 +741,47 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1067,67 +1092,67 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AQ35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="12.6"/>
   <cols>
-    <col min="1" max="1" width="70.453125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="22.26953125" style="1" customWidth="1"/>
-    <col min="3" max="8" width="18.7265625" style="1" customWidth="1"/>
-    <col min="9" max="43" width="11.453125" customWidth="1"/>
-    <col min="44" max="44" width="10.7265625" style="1" customWidth="1"/>
-    <col min="45" max="16384" width="10.7265625" style="1"/>
+    <col min="1" max="1" width="70.42578125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="22.28515625" style="1" customWidth="1"/>
+    <col min="3" max="8" width="18.7109375" style="1" customWidth="1"/>
+    <col min="9" max="43" width="11.42578125" customWidth="1"/>
+    <col min="44" max="44" width="10.7109375" style="1" customWidth="1"/>
+    <col min="45" max="16384" width="10.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="31" t="s">
+    <row r="1" spans="1:13" ht="39.950000000000003" customHeight="1">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="31" t="s">
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="32"/>
-    </row>
-    <row r="2" spans="1:13" ht="41.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
+      <c r="H1" s="29"/>
+    </row>
+    <row r="2" spans="1:13" ht="41.1" customHeight="1" thickBot="1">
+      <c r="A2" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-    </row>
-    <row r="3" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="46" t="s">
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+    </row>
+    <row r="3" spans="1:13" ht="39.950000000000003" customHeight="1">
+      <c r="A3" s="36" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="38"/>
       <c r="C3" s="38"/>
       <c r="D3" s="38"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="37" t="s">
+      <c r="E3" s="39"/>
+      <c r="F3" s="32" t="s">
         <v>4</v>
       </c>
       <c r="G3" s="38"/>
-      <c r="H3" s="39"/>
+      <c r="H3" s="40"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
-    <row r="4" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="28" t="s">
+    <row r="4" spans="1:13" ht="39.950000000000003" customHeight="1">
+      <c r="A4" s="37" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="29"/>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="30"/>
+      <c r="B4" s="41"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="42"/>
       <c r="F4" s="12" t="s">
         <v>6</v>
       </c>
@@ -1138,23 +1163,23 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="34" t="s">
+    <row r="5" spans="1:13" ht="39.950000000000003" customHeight="1" thickBot="1">
+      <c r="A5" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="35"/>
-      <c r="C5" s="35"/>
-      <c r="D5" s="35"/>
-      <c r="E5" s="35"/>
-      <c r="F5" s="35"/>
-      <c r="G5" s="35"/>
-      <c r="H5" s="36"/>
-    </row>
-    <row r="6" spans="1:13" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="44" t="s">
+      <c r="B5" s="43"/>
+      <c r="C5" s="43"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="44"/>
+    </row>
+    <row r="6" spans="1:13" ht="90" customHeight="1">
+      <c r="A6" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="40" t="s">
+      <c r="B6" s="33" t="s">
         <v>11</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1176,9 +1201,9 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:13" s="2" customFormat="1" ht="325" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" s="2" customFormat="1" ht="324.95" customHeight="1" thickBot="1">
       <c r="A7" s="45"/>
-      <c r="B7" s="41"/>
+      <c r="B7" s="46"/>
       <c r="C7" s="19" t="s">
         <v>18</v>
       </c>
@@ -1197,9 +1222,14 @@
       <c r="H7" s="20" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="42" t="s">
+      <c r="I7" s="47"/>
+      <c r="J7" s="47"/>
+      <c r="K7" s="47"/>
+      <c r="L7" s="47"/>
+      <c r="M7" s="47"/>
+    </row>
+    <row r="8" spans="1:13" s="2" customFormat="1" ht="18" customHeight="1">
+      <c r="A8" s="34" t="s">
         <v>24</v>
       </c>
       <c r="B8" s="38"/>
@@ -1208,9 +1238,14 @@
       <c r="E8" s="38"/>
       <c r="F8" s="38"/>
       <c r="G8" s="38"/>
-      <c r="H8" s="43"/>
-    </row>
-    <row r="9" spans="1:13" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H8" s="39"/>
+      <c r="I8" s="47"/>
+      <c r="J8" s="47"/>
+      <c r="K8" s="47"/>
+      <c r="L8" s="47"/>
+      <c r="M8" s="47"/>
+    </row>
+    <row r="9" spans="1:13" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A9" s="9" t="s">
         <v>25</v>
       </c>
@@ -1229,8 +1264,13 @@
       <c r="F9" s="14"/>
       <c r="G9" s="14"/>
       <c r="H9" s="15"/>
-    </row>
-    <row r="10" spans="1:13" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I9" s="47"/>
+      <c r="J9" s="47"/>
+      <c r="K9" s="47"/>
+      <c r="L9" s="47"/>
+      <c r="M9" s="47"/>
+    </row>
+    <row r="10" spans="1:13" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A10" s="9" t="s">
         <v>28</v>
       </c>
@@ -1251,8 +1291,13 @@
       <c r="H10" s="15" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I10" s="47"/>
+      <c r="J10" s="47"/>
+      <c r="K10" s="47"/>
+      <c r="L10" s="47"/>
+      <c r="M10" s="47"/>
+    </row>
+    <row r="11" spans="1:13" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A11" s="9" t="s">
         <v>30</v>
       </c>
@@ -1269,8 +1314,13 @@
         <v>27</v>
       </c>
       <c r="H11" s="15"/>
-    </row>
-    <row r="12" spans="1:13" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I11" s="47"/>
+      <c r="J11" s="47"/>
+      <c r="K11" s="47"/>
+      <c r="L11" s="47"/>
+      <c r="M11" s="47"/>
+    </row>
+    <row r="12" spans="1:13" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A12" s="9" t="s">
         <v>32</v>
       </c>
@@ -1291,8 +1341,13 @@
       <c r="H12" s="15" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I12" s="47"/>
+      <c r="J12" s="47"/>
+      <c r="K12" s="47"/>
+      <c r="L12" s="47"/>
+      <c r="M12" s="47"/>
+    </row>
+    <row r="13" spans="1:13" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A13" s="9" t="s">
         <v>34</v>
       </c>
@@ -1311,8 +1366,13 @@
       <c r="H13" s="15" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I13" s="47"/>
+      <c r="J13" s="47"/>
+      <c r="K13" s="47"/>
+      <c r="L13" s="47"/>
+      <c r="M13" s="47"/>
+    </row>
+    <row r="14" spans="1:13" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A14" s="9" t="s">
         <v>36</v>
       </c>
@@ -1331,8 +1391,13 @@
         <v>27</v>
       </c>
       <c r="H14" s="15"/>
-    </row>
-    <row r="15" spans="1:13" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I14" s="47"/>
+      <c r="J14" s="47"/>
+      <c r="K14" s="47"/>
+      <c r="L14" s="47"/>
+      <c r="M14" s="47"/>
+    </row>
+    <row r="15" spans="1:13" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A15" s="9" t="s">
         <v>38</v>
       </c>
@@ -1357,8 +1422,13 @@
       <c r="H15" s="15" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="16" spans="1:13" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I15" s="47"/>
+      <c r="J15" s="47"/>
+      <c r="K15" s="47"/>
+      <c r="L15" s="47"/>
+      <c r="M15" s="47"/>
+    </row>
+    <row r="16" spans="1:13" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A16" s="9" t="s">
         <v>40</v>
       </c>
@@ -1381,18 +1451,47 @@
       <c r="H16" s="15" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="17" spans="1:20" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="9"/>
-      <c r="B17" s="8"/>
-      <c r="C17" s="14"/>
+      <c r="I16" s="47"/>
+      <c r="J16" s="47"/>
+      <c r="K16" s="47"/>
+      <c r="L16" s="47"/>
+      <c r="M16" s="47"/>
+    </row>
+    <row r="17" spans="1:20" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
+      <c r="A17" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>27</v>
+      </c>
       <c r="D17" s="14"/>
       <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="15"/>
-    </row>
-    <row r="18" spans="1:20" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F17" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="G17" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="H17" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="I17" s="47"/>
+      <c r="J17" s="47"/>
+      <c r="K17" s="47"/>
+      <c r="L17" s="47"/>
+      <c r="M17" s="47"/>
+      <c r="N17" s="47"/>
+      <c r="O17" s="47"/>
+      <c r="P17" s="47"/>
+      <c r="Q17" s="47"/>
+      <c r="R17" s="47"/>
+      <c r="S17" s="47"/>
+      <c r="T17" s="47"/>
+    </row>
+    <row r="18" spans="1:20" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A18" s="9"/>
       <c r="B18" s="8"/>
       <c r="C18" s="14"/>
@@ -1401,25 +1500,49 @@
       <c r="F18" s="14"/>
       <c r="G18" s="14"/>
       <c r="H18" s="15"/>
-    </row>
-    <row r="19" spans="1:20" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="33" t="s">
-        <v>43</v>
-      </c>
-      <c r="B19" s="29"/>
-      <c r="C19" s="29"/>
-      <c r="D19" s="29"/>
-      <c r="E19" s="29"/>
-      <c r="F19" s="29"/>
-      <c r="G19" s="29"/>
-      <c r="H19" s="30"/>
-    </row>
-    <row r="20" spans="1:20" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I18" s="47"/>
+      <c r="J18" s="47"/>
+      <c r="K18" s="47"/>
+      <c r="L18" s="47"/>
+      <c r="M18" s="47"/>
+      <c r="N18" s="47"/>
+      <c r="O18" s="47"/>
+      <c r="P18" s="47"/>
+      <c r="Q18" s="47"/>
+      <c r="R18" s="47"/>
+      <c r="S18" s="47"/>
+      <c r="T18" s="47"/>
+    </row>
+    <row r="19" spans="1:20" s="2" customFormat="1" ht="18" customHeight="1">
+      <c r="A19" s="30" t="s">
+        <v>45</v>
+      </c>
+      <c r="B19" s="41"/>
+      <c r="C19" s="41"/>
+      <c r="D19" s="41"/>
+      <c r="E19" s="41"/>
+      <c r="F19" s="41"/>
+      <c r="G19" s="41"/>
+      <c r="H19" s="42"/>
+      <c r="I19" s="47"/>
+      <c r="J19" s="47"/>
+      <c r="K19" s="47"/>
+      <c r="L19" s="47"/>
+      <c r="M19" s="47"/>
+      <c r="N19" s="47"/>
+      <c r="O19" s="47"/>
+      <c r="P19" s="47"/>
+      <c r="Q19" s="47"/>
+      <c r="R19" s="47"/>
+      <c r="S19" s="47"/>
+      <c r="T19" s="47"/>
+    </row>
+    <row r="20" spans="1:20" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A20" s="25" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B20" s="26" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C20" s="14"/>
       <c r="D20" s="27" t="s">
@@ -1429,13 +1552,25 @@
       <c r="F20" s="14"/>
       <c r="G20" s="14"/>
       <c r="H20" s="15"/>
-    </row>
-    <row r="21" spans="1:20" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I20" s="47"/>
+      <c r="J20" s="47"/>
+      <c r="K20" s="47"/>
+      <c r="L20" s="47"/>
+      <c r="M20" s="47"/>
+      <c r="N20" s="47"/>
+      <c r="O20" s="47"/>
+      <c r="P20" s="47"/>
+      <c r="Q20" s="47"/>
+      <c r="R20" s="47"/>
+      <c r="S20" s="47"/>
+      <c r="T20" s="47"/>
+    </row>
+    <row r="21" spans="1:20" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A21" s="25" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B21" s="26" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C21" s="27" t="s">
         <v>27</v>
@@ -1445,13 +1580,25 @@
       <c r="F21" s="14"/>
       <c r="G21" s="14"/>
       <c r="H21" s="15"/>
-    </row>
-    <row r="22" spans="1:20" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I21" s="47"/>
+      <c r="J21" s="47"/>
+      <c r="K21" s="47"/>
+      <c r="L21" s="47"/>
+      <c r="M21" s="47"/>
+      <c r="N21" s="47"/>
+      <c r="O21" s="47"/>
+      <c r="P21" s="47"/>
+      <c r="Q21" s="47"/>
+      <c r="R21" s="47"/>
+      <c r="S21" s="47"/>
+      <c r="T21" s="47"/>
+    </row>
+    <row r="22" spans="1:20" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A22" s="25" t="s">
+        <v>49</v>
+      </c>
+      <c r="B22" s="26" t="s">
         <v>47</v>
-      </c>
-      <c r="B22" s="26" t="s">
-        <v>45</v>
       </c>
       <c r="C22" s="27" t="s">
         <v>27</v>
@@ -1463,8 +1610,20 @@
         <v>27</v>
       </c>
       <c r="H22" s="15"/>
-    </row>
-    <row r="23" spans="1:20" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I22" s="47"/>
+      <c r="J22" s="47"/>
+      <c r="K22" s="47"/>
+      <c r="L22" s="47"/>
+      <c r="M22" s="47"/>
+      <c r="N22" s="47"/>
+      <c r="O22" s="47"/>
+      <c r="P22" s="47"/>
+      <c r="Q22" s="47"/>
+      <c r="R22" s="47"/>
+      <c r="S22" s="47"/>
+      <c r="T22" s="47"/>
+    </row>
+    <row r="23" spans="1:20" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A23" s="9"/>
       <c r="B23" s="8"/>
       <c r="C23" s="14"/>
@@ -1473,8 +1632,20 @@
       <c r="F23" s="14"/>
       <c r="G23" s="14"/>
       <c r="H23" s="15"/>
-    </row>
-    <row r="24" spans="1:20" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I23" s="47"/>
+      <c r="J23" s="47"/>
+      <c r="K23" s="47"/>
+      <c r="L23" s="47"/>
+      <c r="M23" s="47"/>
+      <c r="N23" s="47"/>
+      <c r="O23" s="47"/>
+      <c r="P23" s="47"/>
+      <c r="Q23" s="47"/>
+      <c r="R23" s="47"/>
+      <c r="S23" s="47"/>
+      <c r="T23" s="47"/>
+    </row>
+    <row r="24" spans="1:20" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A24" s="9"/>
       <c r="B24" s="8"/>
       <c r="C24" s="14"/>
@@ -1483,8 +1654,20 @@
       <c r="F24" s="14"/>
       <c r="G24" s="14"/>
       <c r="H24" s="15"/>
-    </row>
-    <row r="25" spans="1:20" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I24" s="47"/>
+      <c r="J24" s="47"/>
+      <c r="K24" s="47"/>
+      <c r="L24" s="47"/>
+      <c r="M24" s="47"/>
+      <c r="N24" s="47"/>
+      <c r="O24" s="47"/>
+      <c r="P24" s="47"/>
+      <c r="Q24" s="47"/>
+      <c r="R24" s="47"/>
+      <c r="S24" s="47"/>
+      <c r="T24" s="47"/>
+    </row>
+    <row r="25" spans="1:20" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A25" s="9"/>
       <c r="B25" s="8"/>
       <c r="C25" s="14"/>
@@ -1493,8 +1676,20 @@
       <c r="F25" s="14"/>
       <c r="G25" s="14"/>
       <c r="H25" s="15"/>
-    </row>
-    <row r="26" spans="1:20" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I25" s="47"/>
+      <c r="J25" s="47"/>
+      <c r="K25" s="47"/>
+      <c r="L25" s="47"/>
+      <c r="M25" s="47"/>
+      <c r="N25" s="47"/>
+      <c r="O25" s="47"/>
+      <c r="P25" s="47"/>
+      <c r="Q25" s="47"/>
+      <c r="R25" s="47"/>
+      <c r="S25" s="47"/>
+      <c r="T25" s="47"/>
+    </row>
+    <row r="26" spans="1:20" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A26" s="9"/>
       <c r="B26" s="8"/>
       <c r="C26" s="14"/>
@@ -1503,20 +1698,44 @@
       <c r="F26" s="14"/>
       <c r="G26" s="14"/>
       <c r="H26" s="15"/>
-    </row>
-    <row r="27" spans="1:20" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="33" t="s">
-        <v>48</v>
-      </c>
-      <c r="B27" s="29"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="29"/>
-      <c r="F27" s="29"/>
-      <c r="G27" s="29"/>
-      <c r="H27" s="30"/>
-    </row>
-    <row r="28" spans="1:20" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I26" s="47"/>
+      <c r="J26" s="47"/>
+      <c r="K26" s="47"/>
+      <c r="L26" s="47"/>
+      <c r="M26" s="47"/>
+      <c r="N26" s="47"/>
+      <c r="O26" s="47"/>
+      <c r="P26" s="47"/>
+      <c r="Q26" s="47"/>
+      <c r="R26" s="47"/>
+      <c r="S26" s="47"/>
+      <c r="T26" s="47"/>
+    </row>
+    <row r="27" spans="1:20" s="2" customFormat="1" ht="18" customHeight="1">
+      <c r="A27" s="30" t="s">
+        <v>50</v>
+      </c>
+      <c r="B27" s="41"/>
+      <c r="C27" s="41"/>
+      <c r="D27" s="41"/>
+      <c r="E27" s="41"/>
+      <c r="F27" s="41"/>
+      <c r="G27" s="41"/>
+      <c r="H27" s="42"/>
+      <c r="I27" s="47"/>
+      <c r="J27" s="47"/>
+      <c r="K27" s="47"/>
+      <c r="L27" s="47"/>
+      <c r="M27" s="47"/>
+      <c r="N27" s="47"/>
+      <c r="O27" s="47"/>
+      <c r="P27" s="47"/>
+      <c r="Q27" s="47"/>
+      <c r="R27" s="47"/>
+      <c r="S27" s="47"/>
+      <c r="T27" s="47"/>
+    </row>
+    <row r="28" spans="1:20" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A28" s="9"/>
       <c r="B28" s="8"/>
       <c r="C28" s="14"/>
@@ -1525,8 +1744,20 @@
       <c r="F28" s="14"/>
       <c r="G28" s="14"/>
       <c r="H28" s="15"/>
-    </row>
-    <row r="29" spans="1:20" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I28" s="47"/>
+      <c r="J28" s="47"/>
+      <c r="K28" s="47"/>
+      <c r="L28" s="47"/>
+      <c r="M28" s="47"/>
+      <c r="N28" s="47"/>
+      <c r="O28" s="47"/>
+      <c r="P28" s="47"/>
+      <c r="Q28" s="47"/>
+      <c r="R28" s="47"/>
+      <c r="S28" s="47"/>
+      <c r="T28" s="47"/>
+    </row>
+    <row r="29" spans="1:20" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A29" s="9"/>
       <c r="B29" s="8"/>
       <c r="C29" s="14"/>
@@ -1535,8 +1766,20 @@
       <c r="F29" s="14"/>
       <c r="G29" s="14"/>
       <c r="H29" s="15"/>
-    </row>
-    <row r="30" spans="1:20" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I29" s="47"/>
+      <c r="J29" s="47"/>
+      <c r="K29" s="47"/>
+      <c r="L29" s="47"/>
+      <c r="M29" s="47"/>
+      <c r="N29" s="47"/>
+      <c r="O29" s="47"/>
+      <c r="P29" s="47"/>
+      <c r="Q29" s="47"/>
+      <c r="R29" s="47"/>
+      <c r="S29" s="47"/>
+      <c r="T29" s="47"/>
+    </row>
+    <row r="30" spans="1:20" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A30" s="9"/>
       <c r="B30" s="8"/>
       <c r="C30" s="14"/>
@@ -1545,11 +1788,22 @@
       <c r="F30" s="14"/>
       <c r="G30" s="14"/>
       <c r="H30" s="15"/>
+      <c r="I30" s="47"/>
+      <c r="J30" s="47"/>
+      <c r="K30" s="47"/>
+      <c r="L30" s="47"/>
+      <c r="M30" s="47"/>
+      <c r="N30" s="47"/>
+      <c r="O30" s="47"/>
+      <c r="P30" s="47"/>
+      <c r="Q30" s="47"/>
+      <c r="R30" s="47"/>
+      <c r="S30" s="47"/>
       <c r="T30" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="31" spans="1:20" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="31" spans="1:20" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A31" s="9"/>
       <c r="B31" s="8"/>
       <c r="C31" s="14"/>
@@ -1558,8 +1812,20 @@
       <c r="F31" s="14"/>
       <c r="G31" s="14"/>
       <c r="H31" s="15"/>
-    </row>
-    <row r="32" spans="1:20" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I31" s="47"/>
+      <c r="J31" s="47"/>
+      <c r="K31" s="47"/>
+      <c r="L31" s="47"/>
+      <c r="M31" s="47"/>
+      <c r="N31" s="47"/>
+      <c r="O31" s="47"/>
+      <c r="P31" s="47"/>
+      <c r="Q31" s="47"/>
+      <c r="R31" s="47"/>
+      <c r="S31" s="47"/>
+      <c r="T31" s="47"/>
+    </row>
+    <row r="32" spans="1:20" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A32" s="9"/>
       <c r="B32" s="8"/>
       <c r="C32" s="14"/>
@@ -1568,8 +1834,20 @@
       <c r="F32" s="14"/>
       <c r="G32" s="14"/>
       <c r="H32" s="15"/>
-    </row>
-    <row r="33" spans="1:8" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I32" s="47"/>
+      <c r="J32" s="47"/>
+      <c r="K32" s="47"/>
+      <c r="L32" s="47"/>
+      <c r="M32" s="47"/>
+      <c r="N32" s="47"/>
+      <c r="O32" s="47"/>
+      <c r="P32" s="47"/>
+      <c r="Q32" s="47"/>
+      <c r="R32" s="47"/>
+      <c r="S32" s="47"/>
+      <c r="T32" s="47"/>
+    </row>
+    <row r="33" spans="1:8" s="2" customFormat="1" ht="39.950000000000003" customHeight="1">
       <c r="A33" s="9"/>
       <c r="B33" s="8"/>
       <c r="C33" s="14"/>
@@ -1579,7 +1857,7 @@
       <c r="G33" s="14"/>
       <c r="H33" s="15"/>
     </row>
-    <row r="34" spans="1:8" s="2" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1">
       <c r="A34" s="10"/>
       <c r="B34" s="11"/>
       <c r="C34" s="16"/>
@@ -1589,7 +1867,7 @@
       <c r="G34" s="16"/>
       <c r="H34" s="17"/>
     </row>
-    <row r="35" spans="1:8" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" s="2" customFormat="1" ht="15" customHeight="1">
       <c r="A35" s="5"/>
       <c r="B35" s="3"/>
       <c r="C35" s="4"/>

</xml_diff>